<commit_message>
Mileage template: blank guidance rows stay blank (T() on grid lookups), taller item rows
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/GrottLuker-Mileage-Expense-Log-2026.xlsx
+++ b/public/templates/GrottLuker-Mileage-Expense-Log-2026.xlsx
@@ -1349,11 +1349,11 @@
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="24">
-        <f>IFERROR(INDEX(Guide!$E$39:$R$41,1,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$39:$R$41,1,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B20" s="25">
-        <f>IFERROR(INDEX(Guide!$E$44:$R$46,1,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$44:$R$46,1,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C20" s="17" t="n"/>
@@ -1363,11 +1363,11 @@
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="24">
-        <f>IFERROR(INDEX(Guide!$E$39:$R$41,2,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$39:$R$41,2,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B21" s="25">
-        <f>IFERROR(INDEX(Guide!$E$44:$R$46,2,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$44:$R$46,2,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C21" s="17" t="n"/>
@@ -1377,11 +1377,11 @@
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="24">
-        <f>IFERROR(INDEX(Guide!$E$39:$R$41,3,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$39:$R$41,3,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B22" s="25">
-        <f>IFERROR(INDEX(Guide!$E$44:$R$46,3,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$44:$R$46,3,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C22" s="17" t="n"/>
@@ -1422,13 +1422,13 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,1,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,1,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B26" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,1,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,1,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C26" s="28">
@@ -1439,13 +1439,13 @@
       <c r="E26" s="17" t="n"/>
       <c r="F26" s="17" t="n"/>
     </row>
-    <row r="27" ht="18" customHeight="1">
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,2,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,2,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B27" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,2,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,2,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C27" s="28">
@@ -1456,13 +1456,13 @@
       <c r="E27" s="17" t="n"/>
       <c r="F27" s="17" t="n"/>
     </row>
-    <row r="28" ht="18" customHeight="1">
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,3,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,3,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B28" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,3,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,3,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C28" s="28">
@@ -1473,13 +1473,13 @@
       <c r="E28" s="17" t="n"/>
       <c r="F28" s="17" t="n"/>
     </row>
-    <row r="29" ht="18" customHeight="1">
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,4,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,4,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B29" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,4,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,4,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C29" s="28">
@@ -1490,13 +1490,13 @@
       <c r="E29" s="17" t="n"/>
       <c r="F29" s="17" t="n"/>
     </row>
-    <row r="30" ht="18" customHeight="1">
+    <row r="30" ht="28" customHeight="1">
       <c r="A30" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,5,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,5,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B30" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,5,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,5,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C30" s="28">
@@ -1507,13 +1507,13 @@
       <c r="E30" s="17" t="n"/>
       <c r="F30" s="17" t="n"/>
     </row>
-    <row r="31" ht="18" customHeight="1">
+    <row r="31" ht="28" customHeight="1">
       <c r="A31" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,6,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,6,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B31" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,6,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,6,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C31" s="28">
@@ -1524,13 +1524,13 @@
       <c r="E31" s="17" t="n"/>
       <c r="F31" s="17" t="n"/>
     </row>
-    <row r="32" ht="18" customHeight="1">
+    <row r="32" ht="28" customHeight="1">
       <c r="A32" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,7,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,7,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B32" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,7,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,7,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C32" s="28">
@@ -1541,13 +1541,13 @@
       <c r="E32" s="17" t="n"/>
       <c r="F32" s="17" t="n"/>
     </row>
-    <row r="33" ht="18" customHeight="1">
+    <row r="33" ht="28" customHeight="1">
       <c r="A33" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,8,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,8,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B33" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,8,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,8,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C33" s="28">
@@ -1558,13 +1558,13 @@
       <c r="E33" s="17" t="n"/>
       <c r="F33" s="17" t="n"/>
     </row>
-    <row r="34" ht="18" customHeight="1">
+    <row r="34" ht="28" customHeight="1">
       <c r="A34" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,9,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,9,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B34" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,9,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,9,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C34" s="28">
@@ -1575,13 +1575,13 @@
       <c r="E34" s="17" t="n"/>
       <c r="F34" s="17" t="n"/>
     </row>
-    <row r="35" ht="18" customHeight="1">
+    <row r="35" ht="28" customHeight="1">
       <c r="A35" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,10,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,10,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B35" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,10,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,10,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C35" s="28">
@@ -1592,13 +1592,13 @@
       <c r="E35" s="17" t="n"/>
       <c r="F35" s="17" t="n"/>
     </row>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,11,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,11,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B36" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,11,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,11,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C36" s="28">
@@ -1609,13 +1609,13 @@
       <c r="E36" s="17" t="n"/>
       <c r="F36" s="17" t="n"/>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="28" customHeight="1">
       <c r="A37" s="26">
-        <f>IFERROR(INDEX(Guide!$E$11:$R$22,12,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$11:$R$22,12,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B37" s="27">
-        <f>IFERROR(INDEX(Guide!$E$25:$R$36,12,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$25:$R$36,12,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C37" s="28">
@@ -8025,11 +8025,11 @@
     </row>
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="24">
-        <f>IFERROR(INDEX(Guide!$E$39:$R$41,1,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$39:$R$41,1,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B28" s="25">
-        <f>IFERROR(INDEX(Guide!$E$44:$R$46,1,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$44:$R$46,1,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C28" s="17" t="n"/>
@@ -8039,11 +8039,11 @@
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="24">
-        <f>IFERROR(INDEX(Guide!$E$39:$R$41,2,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$39:$R$41,2,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B29" s="25">
-        <f>IFERROR(INDEX(Guide!$E$44:$R$46,2,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$44:$R$46,2,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C29" s="17" t="n"/>
@@ -8053,11 +8053,11 @@
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="24">
-        <f>IFERROR(INDEX(Guide!$E$39:$R$41,3,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$39:$R$41,3,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="B30" s="25">
-        <f>IFERROR(INDEX(Guide!$E$44:$R$46,3,Guide!$B$6),"")</f>
+        <f>T(INDEX(Guide!$E$44:$R$46,3,Guide!$B$6))</f>
         <v/>
       </c>
       <c r="C30" s="17" t="n"/>

</xml_diff>

<commit_message>
Templates: formula band sub-lines no longer get the credit appended twice
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/GrottLuker-Mileage-Expense-Log-2026.xlsx
+++ b/public/templates/GrottLuker-Mileage-Expense-Log-2026.xlsx
@@ -1577,7 +1577,7 @@
       <c r="E3" s="1" t="n"/>
       <c r="F3" s="1" t="n"/>
       <c r="G3" s="3">
-        <f>"Tax year "&amp;'Start here'!$B$12&amp;"   ·   Powered by BlueLine Advisors"   ·   Powered by BlueLine Advisors</f>
+        <f>"Tax year "&amp;'Start here'!$B$12&amp;"   ·   Powered by BlueLine Advisors"</f>
         <v/>
       </c>
     </row>
@@ -3992,7 +3992,7 @@
       <c r="G3" s="1" t="n"/>
       <c r="H3" s="1" t="n"/>
       <c r="I3" s="3">
-        <f>"Tax year "&amp;'Start here'!$B$12&amp;"   ·   Powered by BlueLine Advisors"   ·   Powered by BlueLine Advisors</f>
+        <f>"Tax year "&amp;'Start here'!$B$12&amp;"   ·   Powered by BlueLine Advisors"</f>
         <v/>
       </c>
     </row>
@@ -7609,7 +7609,7 @@
       <c r="D3" s="1" t="n"/>
       <c r="E3" s="1" t="n"/>
       <c r="F3" s="3">
-        <f>"Tax year "&amp;'Start here'!$B$12&amp;"   ·   Powered by BlueLine Advisors"   ·   Powered by BlueLine Advisors</f>
+        <f>"Tax year "&amp;'Start here'!$B$12&amp;"   ·   Powered by BlueLine Advisors"</f>
         <v/>
       </c>
     </row>

</xml_diff>